<commit_message>
fix: incluir anexos y flujo alcanzable en la respuesta de consulta
</commit_message>
<xml_diff>
--- a/backend/data/Protocolos y pasos.xlsx
+++ b/backend/data/Protocolos y pasos.xlsx
@@ -511,10 +511,10 @@
     <t xml:space="preserve">¿Es un adulto? </t>
   </si>
   <si>
-    <t>Si no es asi, seleccionar "No"</t>
-  </si>
-  <si>
-    <t>P0034</t>
+    <t>Si no es así, seleccionar "No"</t>
+  </si>
+  <si>
+    <t>C0034</t>
   </si>
   <si>
     <t>Pide a la persona que tosa. ¿Puede toser?</t>
@@ -1847,7 +1847,7 @@
 P0030</t>
   </si>
   <si>
-    <t>P0034
+    <t>C0034
 P0040</t>
   </si>
   <si>
@@ -2023,7 +2023,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2051,6 +2051,9 @@
     <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
@@ -4449,7 +4452,7 @@
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="5" t="s">
         <v>164</v>
       </c>
       <c r="B40" s="4" t="s">
@@ -4466,7 +4469,7 @@
       </c>
       <c r="F40" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>P0034.png</v>
+        <v>C0034.png</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
@@ -8644,12 +8647,12 @@
       <c r="B39" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C39" s="16" t="s">
         <v>607</v>
       </c>
     </row>
     <row r="40" ht="25.5" customHeight="1">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="5" t="s">
         <v>164</v>
       </c>
       <c r="B40" s="4" t="s">
@@ -8663,7 +8666,7 @@
       <c r="A41" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="5" t="s">
         <v>164</v>
       </c>
       <c r="C41" s="4" t="s">
@@ -8674,7 +8677,7 @@
       <c r="A42" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="5" t="s">
         <v>164</v>
       </c>
       <c r="C42" s="4" t="s">
@@ -9234,7 +9237,7 @@
       <c r="B91" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="C91" s="16" t="s">
+      <c r="C91" s="17" t="s">
         <v>613</v>
       </c>
     </row>
@@ -9366,7 +9369,7 @@
       <c r="B103" s="9" t="s">
         <v>338</v>
       </c>
-      <c r="C103" s="17" t="s">
+      <c r="C103" s="18" t="s">
         <v>614</v>
       </c>
     </row>
@@ -9399,7 +9402,7 @@
       <c r="B106" s="9" t="s">
         <v>347</v>
       </c>
-      <c r="C106" s="17" t="s">
+      <c r="C106" s="18" t="s">
         <v>615</v>
       </c>
     </row>
@@ -9476,7 +9479,7 @@
       <c r="B113" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="C113" s="18" t="s">
+      <c r="C113" s="19" t="s">
         <v>616</v>
       </c>
     </row>
@@ -9553,7 +9556,7 @@
       <c r="B120" s="11" t="s">
         <v>389</v>
       </c>
-      <c r="C120" s="19" t="s">
+      <c r="C120" s="20" t="s">
         <v>617</v>
       </c>
     </row>
@@ -9586,7 +9589,7 @@
       <c r="B123" s="11" t="s">
         <v>398</v>
       </c>
-      <c r="C123" s="19" t="s">
+      <c r="C123" s="20" t="s">
         <v>618</v>
       </c>
     </row>
@@ -9707,7 +9710,7 @@
       <c r="B134" s="12" t="s">
         <v>424</v>
       </c>
-      <c r="C134" s="20" t="s">
+      <c r="C134" s="21" t="s">
         <v>619</v>
       </c>
     </row>
@@ -9795,7 +9798,7 @@
       <c r="B142" s="13" t="s">
         <v>448</v>
       </c>
-      <c r="C142" s="21" t="s">
+      <c r="C142" s="22" t="s">
         <v>619</v>
       </c>
     </row>
@@ -9872,7 +9875,7 @@
       <c r="B149" s="14" t="s">
         <v>469</v>
       </c>
-      <c r="C149" s="22" t="s">
+      <c r="C149" s="23" t="s">
         <v>620</v>
       </c>
     </row>

</xml_diff>